<commit_message>
Updated part list for mouser. Noted parts which got delivered
</commit_message>
<xml_diff>
--- a/Bestellliste_Mouser.xlsx
+++ b/Bestellliste_Mouser.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_d_inverter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E51F874-074D-40D0-A54E-BFF837FB4BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00C2A598-B7BC-4C18-A492-4A059A531ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{4EDDE04E-DF36-49B2-99B2-7DAB17E876F7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{4EDDE04E-DF36-49B2-99B2-7DAB17E876F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="98">
   <si>
     <t>Bauteilnummer</t>
   </si>
@@ -321,6 +321,15 @@
   </si>
   <si>
     <t>Bestellliste bei Mouser</t>
+  </si>
+  <si>
+    <t>Eingetroffen:</t>
+  </si>
+  <si>
+    <t>JA</t>
+  </si>
+  <si>
+    <t>Wurden ausversehen 240 bestellt</t>
   </si>
 </sst>
 </file>
@@ -330,7 +339,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -361,8 +370,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -379,6 +402,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -406,11 +439,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -418,9 +453,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="3"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
     <cellStyle name="40 % - Akzent6" xfId="1" builtinId="51"/>
+    <cellStyle name="Gut" xfId="2" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -733,35 +772,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06030089-E156-4B91-8493-C06DF09A69AD}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" customWidth="1"/>
     <col min="2" max="2" width="56.88671875" customWidth="1"/>
     <col min="3" max="3" width="20.88671875" customWidth="1"/>
     <col min="4" max="4" width="16.33203125" customWidth="1"/>
-    <col min="5" max="5" width="78.77734375" customWidth="1"/>
+    <col min="5" max="5" width="42.21875" customWidth="1"/>
     <col min="6" max="6" width="17.5546875" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="23.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D3">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -783,8 +822,11 @@
       <c r="G4" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -809,8 +851,11 @@
         <f t="shared" ref="H5:H6" si="1">G5*$D$3</f>
         <v>4.3499999999999996</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I5" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -828,15 +873,18 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="G6" s="4">
-        <f t="shared" ref="G6:G50" si="2">F6*C6</f>
+        <f t="shared" ref="G6:G49" si="2">F6*C6</f>
         <v>0.28000000000000003</v>
       </c>
       <c r="H6" s="4">
         <f t="shared" si="1"/>
         <v>4.2</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I6" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -861,8 +909,11 @@
         <f>G7*$D$3</f>
         <v>66.3</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I7" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -884,11 +935,14 @@
         <v>1.6</v>
       </c>
       <c r="H8" s="4">
-        <f t="shared" ref="H8:H50" si="3">G8*$D$3</f>
+        <f t="shared" ref="H8:H49" si="3">G8*$D$3</f>
         <v>24</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I8" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -913,8 +967,11 @@
         <f t="shared" si="3"/>
         <v>83.399999999999991</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I9" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -939,8 +996,11 @@
         <f t="shared" si="3"/>
         <v>158.4</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I10" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -965,8 +1025,11 @@
         <f t="shared" si="3"/>
         <v>20.700000000000003</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I11" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -991,8 +1054,11 @@
         <f t="shared" si="3"/>
         <v>31.200000000000003</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I12" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
@@ -1006,6 +1072,9 @@
         <f t="shared" si="0"/>
         <v>105</v>
       </c>
+      <c r="E13" s="8" t="s">
+        <v>97</v>
+      </c>
       <c r="F13" s="4">
         <v>0.1</v>
       </c>
@@ -1017,8 +1086,11 @@
         <f t="shared" si="3"/>
         <v>10.500000000000002</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I13" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -1043,8 +1115,11 @@
         <f t="shared" si="3"/>
         <v>441</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I14" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1069,8 +1144,11 @@
         <f t="shared" si="3"/>
         <v>102.6</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I15" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
@@ -1095,8 +1173,11 @@
         <f t="shared" si="3"/>
         <v>17.100000000000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I16" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -1121,8 +1202,11 @@
         <f t="shared" si="3"/>
         <v>27</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I17" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
@@ -1147,8 +1231,11 @@
         <f t="shared" si="3"/>
         <v>6.75</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I18" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
@@ -1173,8 +1260,11 @@
         <f t="shared" si="3"/>
         <v>6.75</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I19" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
@@ -1199,8 +1289,11 @@
         <f t="shared" si="3"/>
         <v>6.75</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I20" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
@@ -1225,8 +1318,11 @@
         <f t="shared" si="3"/>
         <v>55.800000000000004</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I21" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1251,8 +1347,11 @@
         <f t="shared" si="3"/>
         <v>160.64999999999998</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I22" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>22</v>
       </c>
@@ -1277,8 +1376,11 @@
         <f t="shared" si="3"/>
         <v>616.79999999999995</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I23" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>23</v>
       </c>
@@ -1303,8 +1405,11 @@
         <f t="shared" si="3"/>
         <v>248.39999999999998</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I24" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>24</v>
       </c>
@@ -1333,7 +1438,7 @@
         <v>612.9</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>25</v>
       </c>
@@ -1358,8 +1463,11 @@
         <f t="shared" si="3"/>
         <v>24.150000000000002</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I26" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
@@ -1385,7 +1493,7 @@
         <v>19.8</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
@@ -1410,8 +1518,11 @@
         <f t="shared" si="3"/>
         <v>246.60000000000002</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I28" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>28</v>
       </c>
@@ -1436,8 +1547,11 @@
         <f t="shared" si="3"/>
         <v>22.5</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I29" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>29</v>
       </c>
@@ -1462,8 +1576,11 @@
         <f t="shared" si="3"/>
         <v>12.600000000000001</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I30" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>30</v>
       </c>
@@ -1488,8 +1605,11 @@
         <f t="shared" si="3"/>
         <v>330.3</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I31" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
@@ -1514,8 +1634,11 @@
         <f t="shared" si="3"/>
         <v>4.5000000000000009</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I32" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>50</v>
       </c>
@@ -1540,8 +1663,11 @@
         <f t="shared" si="3"/>
         <v>25.500000000000004</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I33" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>51</v>
       </c>
@@ -1566,8 +1692,11 @@
         <f t="shared" si="3"/>
         <v>25.500000000000004</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I34" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>32</v>
       </c>
@@ -1592,8 +1721,11 @@
         <f t="shared" si="3"/>
         <v>1.5</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I35" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>33</v>
       </c>
@@ -1618,8 +1750,11 @@
         <f t="shared" si="3"/>
         <v>1.5</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I36" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>34</v>
       </c>
@@ -1644,8 +1779,11 @@
         <f t="shared" si="3"/>
         <v>96</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I37" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>35</v>
       </c>
@@ -1670,8 +1808,11 @@
         <f t="shared" si="3"/>
         <v>30</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I38" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>36</v>
       </c>
@@ -1696,8 +1837,11 @@
         <f t="shared" si="3"/>
         <v>28.5</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I39" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>37</v>
       </c>
@@ -1722,8 +1866,11 @@
         <f t="shared" si="3"/>
         <v>25.2</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I40" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>38</v>
       </c>
@@ -1748,8 +1895,11 @@
         <f t="shared" si="3"/>
         <v>41.4</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I41" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>39</v>
       </c>
@@ -1774,8 +1924,11 @@
         <f t="shared" si="3"/>
         <v>48.6</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I42" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>40</v>
       </c>
@@ -1800,8 +1953,11 @@
         <f t="shared" si="3"/>
         <v>27</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I43" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>41</v>
       </c>
@@ -1826,8 +1982,11 @@
         <f t="shared" si="3"/>
         <v>9.0000000000000018</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I44" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>42</v>
       </c>
@@ -1852,8 +2011,11 @@
         <f t="shared" si="3"/>
         <v>9.0000000000000018</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I45" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>43</v>
       </c>
@@ -1878,8 +2040,11 @@
         <f t="shared" si="3"/>
         <v>9.0000000000000018</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I46" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>44</v>
       </c>
@@ -1904,8 +2069,11 @@
         <f t="shared" si="3"/>
         <v>9.0000000000000018</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I47" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>45</v>
       </c>
@@ -1930,8 +2098,11 @@
         <f t="shared" si="3"/>
         <v>9.0000000000000018</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I48" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>46</v>
       </c>
@@ -1956,8 +2127,11 @@
         <f t="shared" si="3"/>
         <v>9.0000000000000018</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I49" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>47</v>
       </c>
@@ -1982,8 +2156,11 @@
         <f t="shared" ref="H50:H51" si="5">G50*$D$3</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I50" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>48</v>
       </c>
@@ -2008,8 +2185,11 @@
         <f t="shared" si="5"/>
         <v>117.00000000000001</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I51" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="G53" t="s">
         <v>91</v>
       </c>
@@ -2017,7 +2197,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9" ht="18" x14ac:dyDescent="0.35">
       <c r="G54" s="4">
         <f>SUM(G5:G51)</f>
         <v>259.38</v>

</xml_diff>